<commit_message>
fix: align total rows columns with actions header
</commit_message>
<xml_diff>
--- a/backend/prisma/seed-data/account-payable.xlsx
+++ b/backend/prisma/seed-data/account-payable.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ATI-User\Downloads\PCMI-Apps\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder (2)\new-cms\backend\prisma\seed-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3884FBE0-54B7-485E-96A3-BCEA370A8BE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" xr2:uid="{C49568A5-158C-924F-8878-5D75329F86B5}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="24885" windowHeight="14910"/>
   </bookViews>
   <sheets>
     <sheet name="AP" sheetId="44" r:id="rId1"/>
@@ -19,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">AP!$A$3:$V$340</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">AP!$A$2:$V$340</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1999" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2002" uniqueCount="484">
   <si>
     <t>COGS</t>
   </si>
@@ -1486,18 +1485,24 @@
   </si>
   <si>
     <t>PPN Masukan</t>
+  </si>
+  <si>
+    <t>PPn WAPU - 2026</t>
+  </si>
+  <si>
+    <t>WA Yogi 5-Jun-26 : Inv 044/227/PCMI/AR/II/2026 Telkomsel ANO Forum 2024 (Lampung, 24-26 Feb2025) : Rp. 221.286.887 MASUK SALES 2025</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="5">
-    <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="167" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="169" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -1633,39 +1638,39 @@
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
+    <xf numFmtId="165" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="41" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
-    <xf numFmtId="41" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="41" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
@@ -1677,7 +1682,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
@@ -1686,21 +1691,21 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyAlignment="1">
@@ -1716,98 +1721,98 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="3" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="20">
     <cellStyle name="Comma [0]" xfId="1" builtinId="6"/>
-    <cellStyle name="Comma [0] 2" xfId="4" xr:uid="{E206625D-CE92-B946-878E-6AA0829E898C}"/>
-    <cellStyle name="Comma [0] 2 2" xfId="12" xr:uid="{2A804006-5001-5049-84D3-FB258FE2E1AB}"/>
-    <cellStyle name="Comma [0] 2 3" xfId="5" xr:uid="{20A799B3-BE5A-964F-BE1E-1391E29E7052}"/>
-    <cellStyle name="Comma [0] 2 3 2" xfId="10" xr:uid="{6B5DF09C-6668-004E-832C-859692394773}"/>
-    <cellStyle name="Comma [0] 2 3 2 2" xfId="17" xr:uid="{2EC272E1-F154-DE4D-8FFC-1738E0F2B485}"/>
-    <cellStyle name="Comma [0] 3" xfId="9" xr:uid="{DCC47050-EC02-4040-8ED8-306B64C985B1}"/>
-    <cellStyle name="Comma [0] 4" xfId="16" xr:uid="{5B145FB2-4D0A-B249-B369-54ABF0C38C9B}"/>
-    <cellStyle name="Comma 2" xfId="6" xr:uid="{EAAE8118-4A1E-3049-ADC2-FB2BB5557A52}"/>
-    <cellStyle name="Comma 2 2" xfId="7" xr:uid="{B0896BE0-35A1-2F49-8BC0-6D90093B48F4}"/>
-    <cellStyle name="Comma 3" xfId="13" xr:uid="{D01750FA-08E4-0C47-9357-0F62E9D605A3}"/>
-    <cellStyle name="Comma 4" xfId="15" xr:uid="{A2EC2101-5781-AC44-BED5-F1BDBB670F1A}"/>
+    <cellStyle name="Comma [0] 2" xfId="4"/>
+    <cellStyle name="Comma [0] 2 2" xfId="12"/>
+    <cellStyle name="Comma [0] 2 3" xfId="5"/>
+    <cellStyle name="Comma [0] 2 3 2" xfId="10"/>
+    <cellStyle name="Comma [0] 2 3 2 2" xfId="17"/>
+    <cellStyle name="Comma [0] 3" xfId="9"/>
+    <cellStyle name="Comma [0] 4" xfId="16"/>
+    <cellStyle name="Comma 2" xfId="6"/>
+    <cellStyle name="Comma 2 2" xfId="7"/>
+    <cellStyle name="Comma 3" xfId="13"/>
+    <cellStyle name="Comma 4" xfId="15"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2" xr:uid="{3B5401B9-DE75-EB48-9DE0-B2B7DAD183EC}"/>
-    <cellStyle name="Normal 2 2" xfId="8" xr:uid="{54DAEB53-87F6-084C-A87B-7176E7EB83C2}"/>
-    <cellStyle name="Normal 2 3" xfId="19" xr:uid="{FA86753D-0FFC-1948-8EF3-B2B2A5BEC3D7}"/>
-    <cellStyle name="Normal 3" xfId="14" xr:uid="{8B874317-EAD8-D042-9017-3A3DD28E4B28}"/>
-    <cellStyle name="Normal 3 4 2" xfId="11" xr:uid="{B424239B-ED7C-D142-AC4A-5D267E1997FC}"/>
-    <cellStyle name="Normal 3 6" xfId="3" xr:uid="{0DE30895-D5B6-4F42-8773-FC3E05E857CB}"/>
-    <cellStyle name="Normal 3 6 2" xfId="18" xr:uid="{8ECA74BB-2D76-474D-9277-CB573693B101}"/>
+    <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Normal 2 2" xfId="8"/>
+    <cellStyle name="Normal 2 3" xfId="19"/>
+    <cellStyle name="Normal 3" xfId="14"/>
+    <cellStyle name="Normal 3 4 2" xfId="11"/>
+    <cellStyle name="Normal 3 6" xfId="3"/>
+    <cellStyle name="Normal 3 6 2" xfId="18"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2118,37 +2123,37 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE5F47C6-9DB2-EE43-A590-530E996D9E45}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:X349"/>
-  <sheetFormatPr defaultColWidth="9.1875" defaultRowHeight="15.45"/>
+  <dimension ref="A1:X350"/>
+  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="23" style="14" customWidth="1"/>
-    <col min="2" max="2" width="11.1875" style="14" customWidth="1"/>
-    <col min="3" max="3" width="29.3125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="11.21875" style="14" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" style="5" customWidth="1"/>
     <col min="4" max="4" width="67" style="5" customWidth="1"/>
-    <col min="5" max="5" width="21.8125" style="50" customWidth="1"/>
-    <col min="6" max="6" width="18.3125" style="17" customWidth="1"/>
-    <col min="7" max="7" width="19.3125" style="17" customWidth="1"/>
-    <col min="8" max="8" width="27.6875" style="5" customWidth="1"/>
-    <col min="9" max="9" width="65.6875" style="5" customWidth="1"/>
-    <col min="10" max="10" width="2.8125" style="7" customWidth="1"/>
-    <col min="11" max="11" width="20.3125" style="6" customWidth="1"/>
-    <col min="12" max="12" width="18.8125" style="6" customWidth="1"/>
-    <col min="13" max="13" width="20.8125" style="6" customWidth="1"/>
+    <col min="5" max="5" width="21.77734375" style="50" customWidth="1"/>
+    <col min="6" max="6" width="18.33203125" style="17" customWidth="1"/>
+    <col min="7" max="7" width="19.33203125" style="17" customWidth="1"/>
+    <col min="8" max="8" width="27.6640625" style="5" customWidth="1"/>
+    <col min="9" max="9" width="65.6640625" style="5" customWidth="1"/>
+    <col min="10" max="10" width="2.77734375" style="7" customWidth="1"/>
+    <col min="11" max="11" width="20.33203125" style="6" customWidth="1"/>
+    <col min="12" max="12" width="18.77734375" style="6" customWidth="1"/>
+    <col min="13" max="13" width="20.77734375" style="6" customWidth="1"/>
     <col min="14" max="14" width="17" style="6" customWidth="1"/>
-    <col min="15" max="16" width="19.3125" style="6" customWidth="1"/>
+    <col min="15" max="16" width="19.33203125" style="6" customWidth="1"/>
     <col min="17" max="17" width="17" style="6" customWidth="1"/>
-    <col min="18" max="18" width="19.6875" style="6" customWidth="1"/>
-    <col min="19" max="19" width="18.3125" style="6" customWidth="1"/>
-    <col min="20" max="20" width="1.8125" style="6" customWidth="1"/>
-    <col min="21" max="21" width="19.8125" style="6" customWidth="1"/>
-    <col min="22" max="22" width="18.8125" style="6" customWidth="1"/>
-    <col min="23" max="23" width="29.6875" style="27" customWidth="1"/>
-    <col min="24" max="24" width="12.5" style="7" bestFit="1" customWidth="1"/>
-    <col min="25" max="16384" width="9.1875" style="7"/>
+    <col min="18" max="18" width="19.6640625" style="6" customWidth="1"/>
+    <col min="19" max="19" width="18.33203125" style="6" customWidth="1"/>
+    <col min="20" max="20" width="1.77734375" style="6" customWidth="1"/>
+    <col min="21" max="21" width="19.77734375" style="6" customWidth="1"/>
+    <col min="22" max="22" width="18.77734375" style="6" customWidth="1"/>
+    <col min="23" max="23" width="29.6640625" style="27" customWidth="1"/>
+    <col min="24" max="24" width="12.44140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="25" max="16384" width="9.21875" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -2569,7 +2574,7 @@
       </c>
       <c r="W8" s="19"/>
     </row>
-    <row r="9" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="9" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A9" s="23" t="s">
         <v>36</v>
       </c>
@@ -2633,7 +2638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="10" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A10" s="23" t="s">
         <v>36</v>
       </c>
@@ -2697,7 +2702,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="11" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A11" s="23" t="s">
         <v>36</v>
       </c>
@@ -2761,7 +2766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="12" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A12" s="23" t="s">
         <v>36</v>
       </c>
@@ -2825,7 +2830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="13" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A13" s="23" t="s">
         <v>36</v>
       </c>
@@ -2889,7 +2894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="14" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A14" s="42" t="s">
         <v>83</v>
       </c>
@@ -2953,7 +2958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="15" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A15" s="42" t="s">
         <v>83</v>
       </c>
@@ -3017,7 +3022,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="16" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A16" s="42" t="s">
         <v>83</v>
       </c>
@@ -3081,7 +3086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="17" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A17" s="42" t="s">
         <v>83</v>
       </c>
@@ -3145,7 +3150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="18" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A18" s="42" t="s">
         <v>83</v>
       </c>
@@ -3209,7 +3214,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="19" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A19" s="42" t="s">
         <v>83</v>
       </c>
@@ -3273,7 +3278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="20" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A20" s="42" t="s">
         <v>83</v>
       </c>
@@ -3337,7 +3342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="21" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A21" s="42" t="s">
         <v>83</v>
       </c>
@@ -3401,7 +3406,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="22" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A22" s="42" t="s">
         <v>83</v>
       </c>
@@ -3465,7 +3470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="23" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A23" s="42" t="s">
         <v>83</v>
       </c>
@@ -3529,7 +3534,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="24" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A24" s="42" t="s">
         <v>83</v>
       </c>
@@ -3593,7 +3598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="25" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A25" s="42" t="s">
         <v>83</v>
       </c>
@@ -3657,7 +3662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="26" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A26" s="42" t="s">
         <v>83</v>
       </c>
@@ -3721,7 +3726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="27" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A27" s="42" t="s">
         <v>83</v>
       </c>
@@ -3785,7 +3790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="28" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A28" s="42" t="s">
         <v>83</v>
       </c>
@@ -3849,7 +3854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="29" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A29" s="42" t="s">
         <v>83</v>
       </c>
@@ -3913,7 +3918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="30" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A30" s="42" t="s">
         <v>83</v>
       </c>
@@ -3977,7 +3982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="31" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A31" s="42" t="s">
         <v>83</v>
       </c>
@@ -4041,7 +4046,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="32" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A32" s="42" t="s">
         <v>83</v>
       </c>
@@ -4105,7 +4110,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="33" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A33" s="42" t="s">
         <v>83</v>
       </c>
@@ -4169,7 +4174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="34" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A34" s="4" t="s">
         <v>38</v>
       </c>
@@ -4235,7 +4240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="35" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A35" s="42" t="s">
         <v>35</v>
       </c>
@@ -4301,7 +4306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="36" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A36" s="42" t="s">
         <v>35</v>
       </c>
@@ -4367,7 +4372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:23" ht="16" customHeight="1">
+    <row r="37" spans="1:23" ht="15.95" customHeight="1">
       <c r="A37" s="42" t="s">
         <v>39</v>
       </c>
@@ -4432,7 +4437,7 @@
       </c>
       <c r="W37" s="8"/>
     </row>
-    <row r="38" spans="1:23" ht="16" customHeight="1">
+    <row r="38" spans="1:23" ht="15.95" customHeight="1">
       <c r="A38" s="42" t="s">
         <v>39</v>
       </c>
@@ -4497,7 +4502,7 @@
       </c>
       <c r="W38" s="8"/>
     </row>
-    <row r="39" spans="1:23" ht="16" customHeight="1">
+    <row r="39" spans="1:23" ht="15.95" customHeight="1">
       <c r="A39" s="42" t="s">
         <v>39</v>
       </c>
@@ -4562,7 +4567,7 @@
       </c>
       <c r="W39" s="8"/>
     </row>
-    <row r="40" spans="1:23" ht="16" customHeight="1">
+    <row r="40" spans="1:23" ht="15.95" customHeight="1">
       <c r="A40" s="42" t="s">
         <v>39</v>
       </c>
@@ -4627,7 +4632,7 @@
       </c>
       <c r="W40" s="8"/>
     </row>
-    <row r="41" spans="1:23" ht="16" customHeight="1">
+    <row r="41" spans="1:23" ht="15.95" customHeight="1">
       <c r="A41" s="42" t="s">
         <v>39</v>
       </c>
@@ -4692,7 +4697,7 @@
       </c>
       <c r="W41" s="8"/>
     </row>
-    <row r="42" spans="1:23" ht="16" customHeight="1">
+    <row r="42" spans="1:23" ht="15.95" customHeight="1">
       <c r="A42" s="42" t="s">
         <v>39</v>
       </c>
@@ -4757,7 +4762,7 @@
       </c>
       <c r="W42" s="8"/>
     </row>
-    <row r="43" spans="1:23" ht="16" customHeight="1">
+    <row r="43" spans="1:23" ht="15.95" customHeight="1">
       <c r="A43" s="42" t="s">
         <v>39</v>
       </c>
@@ -4822,7 +4827,7 @@
       </c>
       <c r="W43" s="8"/>
     </row>
-    <row r="44" spans="1:23" ht="16" customHeight="1">
+    <row r="44" spans="1:23" ht="15.95" customHeight="1">
       <c r="A44" s="42" t="s">
         <v>39</v>
       </c>
@@ -4887,7 +4892,7 @@
       </c>
       <c r="W44" s="8"/>
     </row>
-    <row r="45" spans="1:23" ht="16" customHeight="1">
+    <row r="45" spans="1:23" ht="15.95" customHeight="1">
       <c r="A45" s="42" t="s">
         <v>39</v>
       </c>
@@ -4952,7 +4957,7 @@
       </c>
       <c r="W45" s="8"/>
     </row>
-    <row r="46" spans="1:23" ht="16" customHeight="1">
+    <row r="46" spans="1:23" ht="15.95" customHeight="1">
       <c r="A46" s="42" t="s">
         <v>39</v>
       </c>
@@ -5017,7 +5022,7 @@
       </c>
       <c r="W46" s="8"/>
     </row>
-    <row r="47" spans="1:23" ht="16" customHeight="1">
+    <row r="47" spans="1:23" ht="15.95" customHeight="1">
       <c r="A47" s="42" t="s">
         <v>39</v>
       </c>
@@ -5082,7 +5087,7 @@
       </c>
       <c r="W47" s="8"/>
     </row>
-    <row r="48" spans="1:23" ht="16" customHeight="1">
+    <row r="48" spans="1:23" ht="15.95" customHeight="1">
       <c r="A48" s="42" t="s">
         <v>39</v>
       </c>
@@ -5147,7 +5152,7 @@
       </c>
       <c r="W48" s="8"/>
     </row>
-    <row r="49" spans="1:24" ht="16" customHeight="1">
+    <row r="49" spans="1:24" ht="15.95" customHeight="1">
       <c r="A49" s="42" t="s">
         <v>39</v>
       </c>
@@ -5212,7 +5217,7 @@
       </c>
       <c r="W49" s="8"/>
     </row>
-    <row r="50" spans="1:24" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="50" spans="1:24" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A50" s="4" t="s">
         <v>39</v>
       </c>
@@ -5279,7 +5284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:24" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="51" spans="1:24" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A51" s="4" t="s">
         <v>39</v>
       </c>
@@ -5346,7 +5351,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:24" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="52" spans="1:24" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A52" s="4" t="s">
         <v>39</v>
       </c>
@@ -5419,7 +5424,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="53" spans="1:24" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="53" spans="1:24" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A53" s="4" t="s">
         <v>39</v>
       </c>
@@ -5492,7 +5497,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="54" spans="1:24" ht="16" customHeight="1">
+    <row r="54" spans="1:24" ht="15.95" customHeight="1">
       <c r="A54" s="42" t="s">
         <v>39</v>
       </c>
@@ -5557,7 +5562,7 @@
       </c>
       <c r="W54" s="8"/>
     </row>
-    <row r="55" spans="1:24" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="55" spans="1:24" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A55" s="4" t="s">
         <v>39</v>
       </c>
@@ -5624,7 +5629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:24" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="56" spans="1:24" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A56" s="4" t="s">
         <v>39</v>
       </c>
@@ -5691,7 +5696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:24" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="57" spans="1:24" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A57" s="4" t="s">
         <v>1</v>
       </c>
@@ -5757,7 +5762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:24" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="58" spans="1:24" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A58" s="23" t="s">
         <v>35</v>
       </c>
@@ -5824,7 +5829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:24" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="59" spans="1:24" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A59" s="23" t="s">
         <v>35</v>
       </c>
@@ -5890,7 +5895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:24" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="60" spans="1:24" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A60" s="23" t="s">
         <v>35</v>
       </c>
@@ -5956,7 +5961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:24" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="61" spans="1:24" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A61" s="23" t="s">
         <v>35</v>
       </c>
@@ -6022,7 +6027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:24" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="62" spans="1:24" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A62" s="23" t="s">
         <v>35</v>
       </c>
@@ -6088,7 +6093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:24" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="63" spans="1:24" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A63" s="23" t="s">
         <v>35</v>
       </c>
@@ -6154,7 +6159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:24" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="64" spans="1:24" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A64" s="23" t="s">
         <v>35</v>
       </c>
@@ -6220,7 +6225,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="65" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A65" s="23" t="s">
         <v>35</v>
       </c>
@@ -6286,7 +6291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="66" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A66" s="23" t="s">
         <v>35</v>
       </c>
@@ -6352,7 +6357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="67" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A67" s="42" t="s">
         <v>35</v>
       </c>
@@ -6418,7 +6423,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="68" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A68" s="23" t="s">
         <v>35</v>
       </c>
@@ -6484,7 +6489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="69" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A69" s="23" t="s">
         <v>35</v>
       </c>
@@ -6550,7 +6555,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="70" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A70" s="23" t="s">
         <v>35</v>
       </c>
@@ -6616,7 +6621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="71" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A71" s="23" t="s">
         <v>35</v>
       </c>
@@ -6682,7 +6687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="72" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A72" s="42" t="s">
         <v>35</v>
       </c>
@@ -6748,7 +6753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="73" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A73" s="4" t="s">
         <v>1</v>
       </c>
@@ -6814,7 +6819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="74" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A74" s="4" t="s">
         <v>7</v>
       </c>
@@ -6886,7 +6891,7 @@
         <v>250000000</v>
       </c>
     </row>
-    <row r="75" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="75" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A75" s="4" t="s">
         <v>7</v>
       </c>
@@ -6954,7 +6959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="76" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A76" s="4" t="s">
         <v>7</v>
       </c>
@@ -7022,7 +7027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="77" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A77" s="4" t="s">
         <v>7</v>
       </c>
@@ -7090,7 +7095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="78" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A78" s="4" t="s">
         <v>7</v>
       </c>
@@ -7158,7 +7163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="79" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A79" s="4" t="s">
         <v>7</v>
       </c>
@@ -7226,7 +7231,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="80" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A80" s="4" t="s">
         <v>7</v>
       </c>
@@ -7294,7 +7299,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="81" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A81" s="4" t="s">
         <v>7</v>
       </c>
@@ -7362,7 +7367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="82" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A82" s="4" t="s">
         <v>7</v>
       </c>
@@ -7430,7 +7435,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="83" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A83" s="4" t="s">
         <v>7</v>
       </c>
@@ -7498,7 +7503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="84" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A84" s="4" t="s">
         <v>7</v>
       </c>
@@ -7566,7 +7571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="85" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A85" s="4" t="s">
         <v>7</v>
       </c>
@@ -7634,7 +7639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="86" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A86" s="4" t="s">
         <v>7</v>
       </c>
@@ -7702,7 +7707,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="87" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A87" s="4" t="s">
         <v>7</v>
       </c>
@@ -7770,7 +7775,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="88" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A88" s="4" t="s">
         <v>7</v>
       </c>
@@ -7838,7 +7843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="89" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A89" s="4" t="s">
         <v>7</v>
       </c>
@@ -7906,7 +7911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="90" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A90" s="4" t="s">
         <v>7</v>
       </c>
@@ -7974,7 +7979,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="91" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A91" s="4" t="s">
         <v>7</v>
       </c>
@@ -8042,7 +8047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="92" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A92" s="4" t="s">
         <v>7</v>
       </c>
@@ -8110,7 +8115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="93" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A93" s="4" t="s">
         <v>7</v>
       </c>
@@ -8178,7 +8183,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="94" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A94" s="4" t="s">
         <v>7</v>
       </c>
@@ -8246,7 +8251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="95" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A95" s="4" t="s">
         <v>7</v>
       </c>
@@ -8314,7 +8319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="96" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A96" s="4" t="s">
         <v>7</v>
       </c>
@@ -8382,7 +8387,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="97" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A97" s="4" t="s">
         <v>7</v>
       </c>
@@ -8450,7 +8455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="98" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A98" s="4" t="s">
         <v>7</v>
       </c>
@@ -8518,7 +8523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="99" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A99" s="4" t="s">
         <v>7</v>
       </c>
@@ -8586,7 +8591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="100" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A100" s="4" t="s">
         <v>7</v>
       </c>
@@ -8654,7 +8659,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="101" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A101" s="4" t="s">
         <v>7</v>
       </c>
@@ -8722,7 +8727,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="102" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A102" s="4" t="s">
         <v>7</v>
       </c>
@@ -8790,7 +8795,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="103" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A103" s="4" t="s">
         <v>7</v>
       </c>
@@ -8858,7 +8863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="104" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A104" s="4" t="s">
         <v>7</v>
       </c>
@@ -8926,7 +8931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="105" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A105" s="4" t="s">
         <v>7</v>
       </c>
@@ -8994,7 +8999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="106" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A106" s="4" t="s">
         <v>7</v>
       </c>
@@ -9062,7 +9067,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="107" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A107" s="4" t="s">
         <v>7</v>
       </c>
@@ -9130,7 +9135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="108" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A108" s="4" t="s">
         <v>7</v>
       </c>
@@ -9198,7 +9203,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="109" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A109" s="4" t="s">
         <v>7</v>
       </c>
@@ -9266,7 +9271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="110" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A110" s="4" t="s">
         <v>7</v>
       </c>
@@ -9334,7 +9339,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="111" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A111" s="4" t="s">
         <v>7</v>
       </c>
@@ -9402,7 +9407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="112" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A112" s="4" t="s">
         <v>7</v>
       </c>
@@ -9470,7 +9475,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="113" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A113" s="4" t="s">
         <v>7</v>
       </c>
@@ -9538,7 +9543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="114" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A114" s="4" t="s">
         <v>7</v>
       </c>
@@ -9606,7 +9611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="115" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A115" s="4" t="s">
         <v>7</v>
       </c>
@@ -9674,7 +9679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="116" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A116" s="4" t="s">
         <v>7</v>
       </c>
@@ -9742,7 +9747,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="117" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A117" s="4" t="s">
         <v>7</v>
       </c>
@@ -9810,7 +9815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="118" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A118" s="4" t="s">
         <v>7</v>
       </c>
@@ -9878,7 +9883,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="119" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A119" s="4" t="s">
         <v>7</v>
       </c>
@@ -9946,7 +9951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="120" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A120" s="4" t="s">
         <v>7</v>
       </c>
@@ -10014,7 +10019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="121" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A121" s="4" t="s">
         <v>7</v>
       </c>
@@ -10082,7 +10087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="122" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A122" s="4" t="s">
         <v>7</v>
       </c>
@@ -10150,7 +10155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="123" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A123" s="4" t="s">
         <v>7</v>
       </c>
@@ -10218,7 +10223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="124" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A124" s="4" t="s">
         <v>7</v>
       </c>
@@ -10286,7 +10291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="125" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A125" s="4" t="s">
         <v>7</v>
       </c>
@@ -10354,7 +10359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="126" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A126" s="58" t="s">
         <v>7</v>
       </c>
@@ -10423,7 +10428,7 @@
       </c>
       <c r="W126" s="32"/>
     </row>
-    <row r="127" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="127" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A127" s="58" t="s">
         <v>7</v>
       </c>
@@ -10492,7 +10497,7 @@
       </c>
       <c r="W127" s="32"/>
     </row>
-    <row r="128" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="128" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A128" s="58" t="s">
         <v>7</v>
       </c>
@@ -10561,7 +10566,7 @@
       </c>
       <c r="W128" s="32"/>
     </row>
-    <row r="129" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="129" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A129" s="58" t="s">
         <v>7</v>
       </c>
@@ -10630,7 +10635,7 @@
       </c>
       <c r="W129" s="32"/>
     </row>
-    <row r="130" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="130" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A130" s="58" t="s">
         <v>7</v>
       </c>
@@ -10699,7 +10704,7 @@
       </c>
       <c r="W130" s="32"/>
     </row>
-    <row r="131" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="131" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A131" s="58" t="s">
         <v>7</v>
       </c>
@@ -10768,7 +10773,7 @@
       </c>
       <c r="W131" s="32"/>
     </row>
-    <row r="132" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="132" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A132" s="4" t="s">
         <v>7</v>
       </c>
@@ -10836,7 +10841,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="133" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A133" s="4" t="s">
         <v>7</v>
       </c>
@@ -10904,7 +10909,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="134" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A134" s="4" t="s">
         <v>7</v>
       </c>
@@ -10975,7 +10980,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="135" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="135" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A135" s="4" t="s">
         <v>7</v>
       </c>
@@ -11043,7 +11048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="136" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A136" s="4" t="s">
         <v>7</v>
       </c>
@@ -11111,7 +11116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="137" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A137" s="4" t="s">
         <v>7</v>
       </c>
@@ -11179,7 +11184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="138" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A138" s="4" t="s">
         <v>7</v>
       </c>
@@ -11247,7 +11252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="139" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A139" s="4" t="s">
         <v>7</v>
       </c>
@@ -11315,7 +11320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="140" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A140" s="4" t="s">
         <v>7</v>
       </c>
@@ -11383,7 +11388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="141" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A141" s="4" t="s">
         <v>7</v>
       </c>
@@ -11451,7 +11456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="142" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A142" s="4" t="s">
         <v>7</v>
       </c>
@@ -11519,7 +11524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="143" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A143" s="4" t="s">
         <v>7</v>
       </c>
@@ -11587,7 +11592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="144" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A144" s="4" t="s">
         <v>7</v>
       </c>
@@ -11655,7 +11660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="145" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A145" s="4" t="s">
         <v>7</v>
       </c>
@@ -11723,7 +11728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="146" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A146" s="4" t="s">
         <v>7</v>
       </c>
@@ -11791,7 +11796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="147" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A147" s="4" t="s">
         <v>7</v>
       </c>
@@ -11859,7 +11864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="148" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A148" s="4" t="s">
         <v>7</v>
       </c>
@@ -11927,7 +11932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="149" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A149" s="4" t="s">
         <v>7</v>
       </c>
@@ -11995,7 +12000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="150" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A150" s="4" t="s">
         <v>7</v>
       </c>
@@ -12063,7 +12068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="151" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A151" s="4" t="s">
         <v>7</v>
       </c>
@@ -12131,7 +12136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="152" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A152" s="4" t="s">
         <v>7</v>
       </c>
@@ -12199,7 +12204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="153" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A153" s="4" t="s">
         <v>7</v>
       </c>
@@ -12267,7 +12272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="154" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A154" s="4" t="s">
         <v>7</v>
       </c>
@@ -12335,7 +12340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="155" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A155" s="4" t="s">
         <v>7</v>
       </c>
@@ -12403,7 +12408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="156" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A156" s="4" t="s">
         <v>7</v>
       </c>
@@ -12471,7 +12476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="157" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A157" s="4" t="s">
         <v>7</v>
       </c>
@@ -12539,7 +12544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="158" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A158" s="4" t="s">
         <v>7</v>
       </c>
@@ -12607,7 +12612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="159" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A159" s="4" t="s">
         <v>7</v>
       </c>
@@ -12675,7 +12680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="160" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A160" s="4" t="s">
         <v>1</v>
       </c>
@@ -12743,7 +12748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="161" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A161" s="4" t="s">
         <v>1</v>
       </c>
@@ -12811,7 +12816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="162" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A162" s="4" t="s">
         <v>1</v>
       </c>
@@ -12879,7 +12884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="163" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A163" s="4" t="s">
         <v>1</v>
       </c>
@@ -12947,7 +12952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="164" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A164" s="4" t="s">
         <v>1</v>
       </c>
@@ -13013,7 +13018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="165" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A165" s="4" t="s">
         <v>1</v>
       </c>
@@ -13079,7 +13084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="166" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A166" s="4" t="s">
         <v>1</v>
       </c>
@@ -13147,7 +13152,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="167" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A167" s="4" t="s">
         <v>1</v>
       </c>
@@ -13215,7 +13220,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="168" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A168" s="4" t="s">
         <v>1</v>
       </c>
@@ -13283,7 +13288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="169" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A169" s="4" t="s">
         <v>1</v>
       </c>
@@ -13351,7 +13356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="170" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A170" s="4" t="s">
         <v>1</v>
       </c>
@@ -13419,7 +13424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="171" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A171" s="4" t="s">
         <v>1</v>
       </c>
@@ -13487,7 +13492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="172" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A172" s="4" t="s">
         <v>1</v>
       </c>
@@ -13555,7 +13560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="173" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A173" s="4" t="s">
         <v>1</v>
       </c>
@@ -13623,7 +13628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="174" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A174" s="4" t="s">
         <v>1</v>
       </c>
@@ -13691,7 +13696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="175" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A175" s="4" t="s">
         <v>1</v>
       </c>
@@ -13759,7 +13764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="176" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A176" s="4" t="s">
         <v>1</v>
       </c>
@@ -13827,7 +13832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="177" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A177" s="4" t="s">
         <v>1</v>
       </c>
@@ -13895,7 +13900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="178" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A178" s="4" t="s">
         <v>1</v>
       </c>
@@ -13963,7 +13968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="179" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A179" s="4" t="s">
         <v>1</v>
       </c>
@@ -14031,7 +14036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="180" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A180" s="4" t="s">
         <v>1</v>
       </c>
@@ -14099,7 +14104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="181" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A181" s="4" t="s">
         <v>1</v>
       </c>
@@ -14167,7 +14172,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="182" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A182" s="4" t="s">
         <v>1</v>
       </c>
@@ -14235,7 +14240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="183" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A183" s="4" t="s">
         <v>1</v>
       </c>
@@ -14303,7 +14308,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="184" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A184" s="4" t="s">
         <v>1</v>
       </c>
@@ -14371,7 +14376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="185" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A185" s="4" t="s">
         <v>1</v>
       </c>
@@ -14439,7 +14444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="186" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A186" s="4" t="s">
         <v>1</v>
       </c>
@@ -14507,7 +14512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="187" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A187" s="4" t="s">
         <v>1</v>
       </c>
@@ -14575,7 +14580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="188" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A188" s="4" t="s">
         <v>1</v>
       </c>
@@ -14643,7 +14648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="189" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A189" s="4" t="s">
         <v>1</v>
       </c>
@@ -14711,7 +14716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="190" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A190" s="4" t="s">
         <v>1</v>
       </c>
@@ -14779,7 +14784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="191" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A191" s="4" t="s">
         <v>1</v>
       </c>
@@ -14847,7 +14852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="192" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A192" s="4" t="s">
         <v>1</v>
       </c>
@@ -14915,7 +14920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="193" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A193" s="4" t="s">
         <v>1</v>
       </c>
@@ -14983,7 +14988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="194" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A194" s="4" t="s">
         <v>1</v>
       </c>
@@ -15051,7 +15056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="195" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A195" s="4" t="s">
         <v>1</v>
       </c>
@@ -15119,7 +15124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="196" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A196" s="4" t="s">
         <v>1</v>
       </c>
@@ -15187,7 +15192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="197" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A197" s="4" t="s">
         <v>1</v>
       </c>
@@ -15255,7 +15260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="198" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A198" s="4" t="s">
         <v>1</v>
       </c>
@@ -15323,7 +15328,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="199" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A199" s="4" t="s">
         <v>1</v>
       </c>
@@ -15391,7 +15396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="200" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A200" s="4" t="s">
         <v>1</v>
       </c>
@@ -15459,7 +15464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="201" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A201" s="4" t="s">
         <v>1</v>
       </c>
@@ -15527,7 +15532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="202" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A202" s="4" t="s">
         <v>1</v>
       </c>
@@ -15595,7 +15600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="203" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A203" s="4" t="s">
         <v>1</v>
       </c>
@@ -15663,7 +15668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="204" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A204" s="4" t="s">
         <v>1</v>
       </c>
@@ -15731,7 +15736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="205" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A205" s="4" t="s">
         <v>1</v>
       </c>
@@ -15799,7 +15804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="206" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A206" s="4" t="s">
         <v>1</v>
       </c>
@@ -15867,7 +15872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="207" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A207" s="4" t="s">
         <v>1</v>
       </c>
@@ -15935,7 +15940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="208" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A208" s="4" t="s">
         <v>1</v>
       </c>
@@ -16003,7 +16008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="209" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A209" s="4" t="s">
         <v>1</v>
       </c>
@@ -16071,7 +16076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="210" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A210" s="4" t="s">
         <v>1</v>
       </c>
@@ -16139,7 +16144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="211" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A211" s="4" t="s">
         <v>1</v>
       </c>
@@ -16207,7 +16212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="212" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A212" s="4" t="s">
         <v>1</v>
       </c>
@@ -16275,7 +16280,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="213" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A213" s="4" t="s">
         <v>1</v>
       </c>
@@ -16343,7 +16348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="214" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A214" s="4" t="s">
         <v>1</v>
       </c>
@@ -16411,7 +16416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="215" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A215" s="4" t="s">
         <v>1</v>
       </c>
@@ -16479,7 +16484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="216" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A216" s="4" t="s">
         <v>1</v>
       </c>
@@ -16547,7 +16552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="217" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A217" s="4" t="s">
         <v>1</v>
       </c>
@@ -16615,7 +16620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="218" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A218" s="4" t="s">
         <v>1</v>
       </c>
@@ -16683,7 +16688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="219" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A219" s="4" t="s">
         <v>1</v>
       </c>
@@ -16751,7 +16756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="220" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A220" s="4" t="s">
         <v>1</v>
       </c>
@@ -16819,7 +16824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="221" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A221" s="4" t="s">
         <v>1</v>
       </c>
@@ -16887,7 +16892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="222" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A222" s="4" t="s">
         <v>1</v>
       </c>
@@ -16955,7 +16960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="223" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A223" s="4" t="s">
         <v>1</v>
       </c>
@@ -17023,7 +17028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="224" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A224" s="4" t="s">
         <v>1</v>
       </c>
@@ -17091,7 +17096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="225" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A225" s="4" t="s">
         <v>1</v>
       </c>
@@ -17159,7 +17164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="226" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A226" s="4" t="s">
         <v>1</v>
       </c>
@@ -17227,7 +17232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="227" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A227" s="4" t="s">
         <v>1</v>
       </c>
@@ -17295,7 +17300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="228" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A228" s="4" t="s">
         <v>1</v>
       </c>
@@ -17363,7 +17368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="229" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A229" s="4" t="s">
         <v>1</v>
       </c>
@@ -17431,7 +17436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="230" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A230" s="4" t="s">
         <v>1</v>
       </c>
@@ -17499,7 +17504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="231" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A231" s="4" t="s">
         <v>1</v>
       </c>
@@ -17567,7 +17572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="232" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A232" s="4" t="s">
         <v>1</v>
       </c>
@@ -17635,7 +17640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="233" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A233" s="4" t="s">
         <v>1</v>
       </c>
@@ -17703,7 +17708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="234" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="234" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A234" s="4" t="s">
         <v>1</v>
       </c>
@@ -17771,7 +17776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="235" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A235" s="4" t="s">
         <v>1</v>
       </c>
@@ -17839,7 +17844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="236" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="236" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A236" s="4" t="s">
         <v>1</v>
       </c>
@@ -17907,7 +17912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="237" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="237" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A237" s="4" t="s">
         <v>1</v>
       </c>
@@ -17975,7 +17980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="238" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A238" s="4" t="s">
         <v>1</v>
       </c>
@@ -18043,7 +18048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="239" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A239" s="4" t="s">
         <v>1</v>
       </c>
@@ -18111,7 +18116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="240" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="240" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A240" s="4" t="s">
         <v>1</v>
       </c>
@@ -18179,7 +18184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="241" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A241" s="4" t="s">
         <v>1</v>
       </c>
@@ -18247,7 +18252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="242" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="242" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A242" s="4" t="s">
         <v>1</v>
       </c>
@@ -18315,7 +18320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="243" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="243" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A243" s="4" t="s">
         <v>1</v>
       </c>
@@ -18383,7 +18388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="244" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="244" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A244" s="4" t="s">
         <v>1</v>
       </c>
@@ -18451,7 +18456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="245" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A245" s="4" t="s">
         <v>1</v>
       </c>
@@ -18519,7 +18524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="246" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="246" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A246" s="4" t="s">
         <v>1</v>
       </c>
@@ -18587,7 +18592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="247" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="247" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A247" s="4" t="s">
         <v>1</v>
       </c>
@@ -18655,7 +18660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="248" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A248" s="4" t="s">
         <v>1</v>
       </c>
@@ -18723,7 +18728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="249" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="249" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A249" s="4" t="s">
         <v>1</v>
       </c>
@@ -18791,7 +18796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="250" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A250" s="4" t="s">
         <v>1</v>
       </c>
@@ -18859,7 +18864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="251" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A251" s="4" t="s">
         <v>1</v>
       </c>
@@ -18927,7 +18932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="252" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="252" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A252" s="4" t="s">
         <v>1</v>
       </c>
@@ -18995,7 +19000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="253" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="253" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A253" s="4" t="s">
         <v>1</v>
       </c>
@@ -19063,7 +19068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="254" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="254" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A254" s="4" t="s">
         <v>1</v>
       </c>
@@ -19131,7 +19136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="255" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A255" s="4" t="s">
         <v>1</v>
       </c>
@@ -19199,7 +19204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="256" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A256" s="4" t="s">
         <v>1</v>
       </c>
@@ -19267,7 +19272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="257" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A257" s="4" t="s">
         <v>1</v>
       </c>
@@ -19335,7 +19340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="258" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A258" s="4" t="s">
         <v>1</v>
       </c>
@@ -19403,7 +19408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="259" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="259" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A259" s="4" t="s">
         <v>1</v>
       </c>
@@ -19471,7 +19476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="260" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A260" s="4" t="s">
         <v>1</v>
       </c>
@@ -19539,7 +19544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="261" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="261" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A261" s="4" t="s">
         <v>1</v>
       </c>
@@ -19607,7 +19612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="262" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="262" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A262" s="4" t="s">
         <v>1</v>
       </c>
@@ -19675,7 +19680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="263" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="263" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A263" s="4" t="s">
         <v>1</v>
       </c>
@@ -19743,7 +19748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="264" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="264" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A264" s="4" t="s">
         <v>1</v>
       </c>
@@ -19811,7 +19816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="265" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="265" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A265" s="4" t="s">
         <v>1</v>
       </c>
@@ -19879,7 +19884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="266" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="266" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A266" s="4" t="s">
         <v>1</v>
       </c>
@@ -19947,7 +19952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="267" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="267" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A267" s="4" t="s">
         <v>1</v>
       </c>
@@ -20015,7 +20020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="268" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="268" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A268" s="4" t="s">
         <v>1</v>
       </c>
@@ -20083,7 +20088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="269" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="269" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A269" s="4" t="s">
         <v>1</v>
       </c>
@@ -20151,7 +20156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="270" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="270" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A270" s="4" t="s">
         <v>1</v>
       </c>
@@ -20219,7 +20224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="271" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="271" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A271" s="4" t="s">
         <v>1</v>
       </c>
@@ -20287,7 +20292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="272" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="272" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A272" s="4" t="s">
         <v>1</v>
       </c>
@@ -20355,7 +20360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="273" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A273" s="4" t="s">
         <v>1</v>
       </c>
@@ -20423,7 +20428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="274" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="274" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A274" s="4" t="s">
         <v>1</v>
       </c>
@@ -20491,7 +20496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="275" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="275" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A275" s="4" t="s">
         <v>1</v>
       </c>
@@ -20559,7 +20564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="276" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="276" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A276" s="4" t="s">
         <v>1</v>
       </c>
@@ -20627,7 +20632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="277" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="277" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A277" s="4" t="s">
         <v>1</v>
       </c>
@@ -20695,7 +20700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="278" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="278" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A278" s="4" t="s">
         <v>1</v>
       </c>
@@ -20763,7 +20768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="279" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="279" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A279" s="4" t="s">
         <v>1</v>
       </c>
@@ -20831,7 +20836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="280" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="280" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A280" s="4" t="s">
         <v>1</v>
       </c>
@@ -20899,7 +20904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="281" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="281" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A281" s="4" t="s">
         <v>1</v>
       </c>
@@ -20967,7 +20972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="282" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="282" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A282" s="4" t="s">
         <v>1</v>
       </c>
@@ -21035,7 +21040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="283" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="283" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A283" s="4" t="s">
         <v>1</v>
       </c>
@@ -21103,7 +21108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="284" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="284" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A284" s="4" t="s">
         <v>1</v>
       </c>
@@ -21171,7 +21176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="285" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="285" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A285" s="4" t="s">
         <v>1</v>
       </c>
@@ -21239,7 +21244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="286" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="286" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A286" s="4" t="s">
         <v>1</v>
       </c>
@@ -21307,7 +21312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="287" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="287" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A287" s="4" t="s">
         <v>1</v>
       </c>
@@ -21375,7 +21380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="288" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="288" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A288" s="4" t="s">
         <v>1</v>
       </c>
@@ -21443,7 +21448,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="289" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="289" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A289" s="4" t="s">
         <v>1</v>
       </c>
@@ -21511,7 +21516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="290" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="290" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A290" s="4" t="s">
         <v>1</v>
       </c>
@@ -21579,7 +21584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="291" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="291" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A291" s="4" t="s">
         <v>1</v>
       </c>
@@ -21647,7 +21652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="292" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="292" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A292" s="4" t="s">
         <v>1</v>
       </c>
@@ -21715,7 +21720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="293" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="293" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A293" s="4" t="s">
         <v>1</v>
       </c>
@@ -21783,7 +21788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="294" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="294" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A294" s="4" t="s">
         <v>1</v>
       </c>
@@ -21851,7 +21856,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="295" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="295" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A295" s="4" t="s">
         <v>1</v>
       </c>
@@ -21919,7 +21924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="296" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="296" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A296" s="4" t="s">
         <v>1</v>
       </c>
@@ -21987,7 +21992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="297" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="297" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A297" s="4" t="s">
         <v>1</v>
       </c>
@@ -22055,7 +22060,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="298" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="298" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A298" s="4" t="s">
         <v>1</v>
       </c>
@@ -22123,7 +22128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="299" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="299" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A299" s="4" t="s">
         <v>1</v>
       </c>
@@ -22191,7 +22196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="300" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="300" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A300" s="4" t="s">
         <v>1</v>
       </c>
@@ -22259,7 +22264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="301" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="301" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A301" s="4" t="s">
         <v>1</v>
       </c>
@@ -22327,7 +22332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="302" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="302" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A302" s="4" t="s">
         <v>1</v>
       </c>
@@ -22395,7 +22400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="303" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="303" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A303" s="4" t="s">
         <v>1</v>
       </c>
@@ -22463,7 +22468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="304" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="304" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A304" s="4" t="s">
         <v>1</v>
       </c>
@@ -22531,7 +22536,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="305" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="305" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A305" s="4" t="s">
         <v>1</v>
       </c>
@@ -22599,7 +22604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="306" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="306" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A306" s="4" t="s">
         <v>1</v>
       </c>
@@ -22667,7 +22672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="307" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="307" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A307" s="4" t="s">
         <v>1</v>
       </c>
@@ -22735,7 +22740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="308" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="308" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A308" s="4" t="s">
         <v>1</v>
       </c>
@@ -22803,7 +22808,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="309" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="309" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A309" s="4" t="s">
         <v>1</v>
       </c>
@@ -22871,7 +22876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="310" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="310" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A310" s="4" t="s">
         <v>1</v>
       </c>
@@ -22939,7 +22944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="311" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="311" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A311" s="4" t="s">
         <v>1</v>
       </c>
@@ -23007,7 +23012,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="312" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="312" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A312" s="4" t="s">
         <v>1</v>
       </c>
@@ -23075,7 +23080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="313" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="313" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A313" s="4" t="s">
         <v>1</v>
       </c>
@@ -23143,7 +23148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="314" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="314" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A314" s="4" t="s">
         <v>1</v>
       </c>
@@ -23211,7 +23216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="315" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="315" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A315" s="4" t="s">
         <v>1</v>
       </c>
@@ -23279,7 +23284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="316" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="316" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A316" s="4" t="s">
         <v>1</v>
       </c>
@@ -23347,7 +23352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="317" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="317" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A317" s="4" t="s">
         <v>1</v>
       </c>
@@ -23415,7 +23420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="318" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="318" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A318" s="4" t="s">
         <v>1</v>
       </c>
@@ -23479,11 +23484,11 @@
         <v>7280000</v>
       </c>
       <c r="V318" s="6">
-        <f t="shared" ref="V318:V340" si="59">G318+S318</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="319" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+        <f t="shared" ref="V318:V341" si="59">G318+S318</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="319" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A319" s="4" t="s">
         <v>1</v>
       </c>
@@ -23551,7 +23556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="320" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="320" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A320" s="4" t="s">
         <v>1</v>
       </c>
@@ -23619,7 +23624,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="321" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="321" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A321" s="4" t="s">
         <v>1</v>
       </c>
@@ -23687,7 +23692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="322" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="322" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A322" s="4" t="s">
         <v>1</v>
       </c>
@@ -23755,7 +23760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="323" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="323" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A323" s="4" t="s">
         <v>1</v>
       </c>
@@ -23823,7 +23828,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="324" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="324" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A324" s="4" t="s">
         <v>1</v>
       </c>
@@ -23891,7 +23896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="325" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="325" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A325" s="4" t="s">
         <v>1</v>
       </c>
@@ -23959,7 +23964,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="326" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="326" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A326" s="4" t="s">
         <v>1</v>
       </c>
@@ -24027,7 +24032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="327" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="327" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A327" s="4" t="s">
         <v>1</v>
       </c>
@@ -24095,7 +24100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="328" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="328" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A328" s="4" t="s">
         <v>1</v>
       </c>
@@ -24163,7 +24168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="329" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="329" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A329" s="4" t="s">
         <v>1</v>
       </c>
@@ -24231,7 +24236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="330" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="330" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A330" s="4" t="s">
         <v>1</v>
       </c>
@@ -24299,7 +24304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="331" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="331" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A331" s="4" t="s">
         <v>1</v>
       </c>
@@ -24367,7 +24372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="332" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="332" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A332" s="4" t="s">
         <v>1</v>
       </c>
@@ -24435,7 +24440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="333" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="333" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A333" s="4" t="s">
         <v>1</v>
       </c>
@@ -24503,7 +24508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="334" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="334" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A334" s="4" t="s">
         <v>1</v>
       </c>
@@ -24571,7 +24576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="335" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="335" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A335" s="4" t="s">
         <v>1</v>
       </c>
@@ -24639,7 +24644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="336" spans="1:22" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="336" spans="1:22" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A336" s="4" t="s">
         <v>1</v>
       </c>
@@ -24707,7 +24712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="337" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="337" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A337" s="4" t="s">
         <v>1</v>
       </c>
@@ -24775,7 +24780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="338" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="338" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A338" s="4" t="s">
         <v>1</v>
       </c>
@@ -24843,7 +24848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="339" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="339" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A339" s="4" t="s">
         <v>1</v>
       </c>
@@ -24911,7 +24916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="340" spans="1:23" s="8" customFormat="1" ht="16" customHeight="1">
+    <row r="340" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
       <c r="A340" s="4" t="s">
         <v>1</v>
       </c>
@@ -24979,230 +24984,291 @@
         <v>0</v>
       </c>
     </row>
-    <row r="342" spans="1:23" s="27" customFormat="1">
-      <c r="A342" s="14"/>
-      <c r="B342" s="14"/>
-      <c r="C342" s="5"/>
-      <c r="D342" s="5"/>
-      <c r="E342" s="50">
-        <f>SUBTOTAL(9,E4:E341)</f>
-        <v>7257557384.8400002</v>
-      </c>
-      <c r="F342" s="50">
-        <f>SUBTOTAL(9,F4:F341)</f>
-        <v>0</v>
-      </c>
-      <c r="G342" s="50">
-        <f>SUBTOTAL(9,G4:G341)</f>
-        <v>0</v>
-      </c>
-      <c r="H342" s="5"/>
-      <c r="I342" s="5"/>
-      <c r="J342" s="7"/>
-      <c r="K342" s="55">
-        <f t="shared" ref="K342:S342" si="68">SUBTOTAL(9,K4:K341)</f>
-        <v>686680889</v>
-      </c>
-      <c r="L342" s="55">
-        <f t="shared" si="68"/>
-        <v>149183884</v>
-      </c>
-      <c r="M342" s="55">
-        <f t="shared" si="68"/>
-        <v>-393065428</v>
-      </c>
-      <c r="N342" s="55">
-        <f t="shared" si="68"/>
-        <v>0</v>
-      </c>
-      <c r="O342" s="55">
-        <f t="shared" si="68"/>
-        <v>-1500000</v>
-      </c>
-      <c r="P342" s="55">
-        <f t="shared" si="68"/>
-        <v>-154034667</v>
-      </c>
-      <c r="Q342" s="55">
-        <f t="shared" si="68"/>
-        <v>-2892500</v>
-      </c>
-      <c r="R342" s="55">
-        <f t="shared" si="68"/>
-        <v>-540844924.84000003</v>
-      </c>
-      <c r="S342" s="55">
-        <f t="shared" si="68"/>
-        <v>-3323562928</v>
-      </c>
-      <c r="T342" s="34"/>
-      <c r="U342" s="55">
-        <f>SUBTOTAL(9,U4:U341)</f>
-        <v>3677521710</v>
-      </c>
-      <c r="V342" s="55">
-        <f>SUBTOTAL(9,V4:V341)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="343" spans="1:23" s="16" customFormat="1">
+    <row r="341" spans="1:23" s="8" customFormat="1" ht="15.95" customHeight="1">
+      <c r="A341" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B341" s="35">
+        <v>2025</v>
+      </c>
+      <c r="C341" s="26" t="s">
+        <v>482</v>
+      </c>
+      <c r="D341" s="29" t="s">
+        <v>483</v>
+      </c>
+      <c r="E341" s="36">
+        <v>21929331</v>
+      </c>
+      <c r="F341" s="6">
+        <v>0</v>
+      </c>
+      <c r="G341" s="6">
+        <v>0</v>
+      </c>
+      <c r="H341" s="5"/>
+      <c r="I341" s="29"/>
+      <c r="J341" s="29"/>
+      <c r="K341" s="6">
+        <v>0</v>
+      </c>
+      <c r="L341" s="6">
+        <v>0</v>
+      </c>
+      <c r="M341" s="6">
+        <v>0</v>
+      </c>
+      <c r="N341" s="6">
+        <v>0</v>
+      </c>
+      <c r="O341" s="6">
+        <v>0</v>
+      </c>
+      <c r="P341" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q341" s="6">
+        <v>0</v>
+      </c>
+      <c r="R341" s="6">
+        <v>0</v>
+      </c>
+      <c r="S341" s="6">
+        <v>0</v>
+      </c>
+      <c r="T341" s="6"/>
+      <c r="U341" s="6">
+        <v>21929331</v>
+      </c>
+      <c r="V341" s="6">
+        <f t="shared" si="59"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="343" spans="1:23" s="27" customFormat="1">
       <c r="A343" s="14"/>
       <c r="B343" s="14"/>
       <c r="C343" s="5"/>
-      <c r="D343" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E343" s="50"/>
-      <c r="F343" s="17"/>
-      <c r="G343" s="17"/>
+      <c r="D343" s="5"/>
+      <c r="E343" s="50">
+        <f>SUBTOTAL(9,E4:E342)</f>
+        <v>7279486715.8400002</v>
+      </c>
+      <c r="F343" s="50">
+        <f>SUBTOTAL(9,F4:F342)</f>
+        <v>0</v>
+      </c>
+      <c r="G343" s="50">
+        <f>SUBTOTAL(9,G4:G342)</f>
+        <v>0</v>
+      </c>
       <c r="H343" s="5"/>
       <c r="I343" s="5"/>
       <c r="J343" s="7"/>
-      <c r="K343" s="6"/>
-      <c r="L343" s="6"/>
-      <c r="M343" s="6"/>
-      <c r="N343" s="6"/>
-      <c r="O343" s="6"/>
-      <c r="P343" s="6"/>
-      <c r="Q343" s="6"/>
-      <c r="R343" s="6"/>
-      <c r="S343" s="6"/>
-      <c r="T343" s="6"/>
-      <c r="U343" s="6"/>
-      <c r="V343" s="6"/>
-      <c r="W343" s="27"/>
-    </row>
-    <row r="344" spans="1:23" s="66" customFormat="1">
-      <c r="A344" s="63"/>
-      <c r="B344" s="63"/>
-      <c r="C344" s="62"/>
-      <c r="D344" s="62"/>
-      <c r="E344" s="64"/>
-      <c r="F344" s="65"/>
-      <c r="G344" s="65"/>
-      <c r="H344" s="62"/>
-      <c r="I344" s="62"/>
-      <c r="K344" s="60">
+      <c r="K343" s="55">
+        <f t="shared" ref="K343:S343" si="68">SUBTOTAL(9,K4:K342)</f>
         <v>686680889</v>
       </c>
-      <c r="L344" s="60">
+      <c r="L343" s="55">
+        <f t="shared" si="68"/>
         <v>149183884</v>
       </c>
-      <c r="M344" s="60">
+      <c r="M343" s="55">
+        <f t="shared" si="68"/>
         <v>-393065428</v>
       </c>
-      <c r="N344" s="60">
-        <v>0</v>
-      </c>
-      <c r="O344" s="60">
+      <c r="N343" s="55">
+        <f t="shared" si="68"/>
+        <v>0</v>
+      </c>
+      <c r="O343" s="55">
+        <f t="shared" si="68"/>
         <v>-1500000</v>
       </c>
-      <c r="P344" s="60">
+      <c r="P343" s="55">
+        <f t="shared" si="68"/>
         <v>-154034667</v>
       </c>
-      <c r="Q344" s="60">
+      <c r="Q343" s="55">
+        <f t="shared" si="68"/>
         <v>-2892500</v>
       </c>
-      <c r="R344" s="60">
+      <c r="R343" s="55">
+        <f t="shared" si="68"/>
+        <v>-540844924.84000003</v>
+      </c>
+      <c r="S343" s="55">
+        <f t="shared" si="68"/>
+        <v>-3323562928</v>
+      </c>
+      <c r="T343" s="34"/>
+      <c r="U343" s="55">
+        <f>SUBTOTAL(9,U4:U342)</f>
+        <v>3699451041</v>
+      </c>
+      <c r="V343" s="55">
+        <f>SUBTOTAL(9,V4:V342)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="344" spans="1:23" s="16" customFormat="1">
+      <c r="A344" s="14"/>
+      <c r="B344" s="14"/>
+      <c r="C344" s="5"/>
+      <c r="D344" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E344" s="50"/>
+      <c r="F344" s="17"/>
+      <c r="G344" s="17"/>
+      <c r="H344" s="5"/>
+      <c r="I344" s="5"/>
+      <c r="J344" s="7"/>
+      <c r="K344" s="6"/>
+      <c r="L344" s="6"/>
+      <c r="M344" s="6"/>
+      <c r="N344" s="6"/>
+      <c r="O344" s="6"/>
+      <c r="P344" s="6"/>
+      <c r="Q344" s="6"/>
+      <c r="R344" s="6"/>
+      <c r="S344" s="6"/>
+      <c r="T344" s="6"/>
+      <c r="U344" s="6"/>
+      <c r="V344" s="6"/>
+      <c r="W344" s="27"/>
+    </row>
+    <row r="345" spans="1:23" s="66" customFormat="1">
+      <c r="A345" s="63"/>
+      <c r="B345" s="63"/>
+      <c r="C345" s="62"/>
+      <c r="D345" s="62"/>
+      <c r="E345" s="64"/>
+      <c r="F345" s="65"/>
+      <c r="G345" s="65"/>
+      <c r="H345" s="62"/>
+      <c r="I345" s="62"/>
+      <c r="K345" s="60">
+        <v>686680889</v>
+      </c>
+      <c r="L345" s="60">
+        <v>149183884</v>
+      </c>
+      <c r="M345" s="60">
+        <v>-393065428</v>
+      </c>
+      <c r="N345" s="60">
+        <v>0</v>
+      </c>
+      <c r="O345" s="60">
+        <v>-1500000</v>
+      </c>
+      <c r="P345" s="60">
+        <v>-154034667</v>
+      </c>
+      <c r="Q345" s="60">
+        <v>-2892500</v>
+      </c>
+      <c r="R345" s="60">
         <v>-540844924.83999991</v>
       </c>
-      <c r="S344" s="60">
-        <v>0</v>
-      </c>
-      <c r="T344" s="60"/>
-      <c r="U344" s="60"/>
-      <c r="V344" s="60"/>
-      <c r="W344" s="27"/>
-    </row>
-    <row r="345" spans="1:23">
-      <c r="L345" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="M345" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="N345" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="O345" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="P345" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q345" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="R345" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="S345" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="346" spans="1:23" s="48" customFormat="1">
-      <c r="A346" s="56"/>
-      <c r="B346" s="56"/>
-      <c r="C346" s="31"/>
-      <c r="D346" s="31"/>
-      <c r="E346" s="57"/>
-      <c r="F346" s="37"/>
-      <c r="G346" s="37"/>
-      <c r="H346" s="31"/>
-      <c r="I346" s="31"/>
-      <c r="K346" s="40">
-        <f t="shared" ref="K346:S346" si="69">K342-K344</f>
-        <v>0</v>
-      </c>
-      <c r="L346" s="40">
+      <c r="S345" s="60">
+        <v>0</v>
+      </c>
+      <c r="T345" s="60"/>
+      <c r="U345" s="60"/>
+      <c r="V345" s="60"/>
+      <c r="W345" s="27"/>
+    </row>
+    <row r="346" spans="1:23">
+      <c r="L346" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="M346" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="N346" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="O346" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="P346" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q346" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="R346" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="S346" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="347" spans="1:23" s="48" customFormat="1">
+      <c r="A347" s="56"/>
+      <c r="B347" s="56"/>
+      <c r="C347" s="31"/>
+      <c r="D347" s="31"/>
+      <c r="E347" s="57"/>
+      <c r="F347" s="37"/>
+      <c r="G347" s="37"/>
+      <c r="H347" s="31"/>
+      <c r="I347" s="31"/>
+      <c r="K347" s="40">
+        <f t="shared" ref="K347:S347" si="69">K343-K345</f>
+        <v>0</v>
+      </c>
+      <c r="L347" s="40">
         <f t="shared" si="69"/>
         <v>0</v>
       </c>
-      <c r="M346" s="40">
+      <c r="M347" s="40">
         <f t="shared" si="69"/>
         <v>0</v>
       </c>
-      <c r="N346" s="40">
+      <c r="N347" s="40">
         <f t="shared" si="69"/>
         <v>0</v>
       </c>
-      <c r="O346" s="40">
+      <c r="O347" s="40">
         <f t="shared" si="69"/>
         <v>0</v>
       </c>
-      <c r="P346" s="40">
+      <c r="P347" s="40">
         <f t="shared" si="69"/>
         <v>0</v>
       </c>
-      <c r="Q346" s="40">
+      <c r="Q347" s="40">
         <f t="shared" si="69"/>
         <v>0</v>
       </c>
-      <c r="R346" s="40">
+      <c r="R347" s="40">
         <f t="shared" si="69"/>
         <v>0</v>
       </c>
-      <c r="S346" s="40">
+      <c r="S347" s="40">
         <f t="shared" si="69"/>
         <v>-3323562928</v>
       </c>
-      <c r="T346" s="40"/>
-      <c r="U346" s="40"/>
-      <c r="V346" s="40"/>
-      <c r="W346" s="41"/>
-    </row>
-    <row r="348" spans="1:23">
-      <c r="R348" s="6" t="s">
-        <v>13</v>
-      </c>
+      <c r="T347" s="40"/>
+      <c r="U347" s="40"/>
+      <c r="V347" s="40"/>
+      <c r="W347" s="41"/>
     </row>
     <row r="349" spans="1:23">
       <c r="R349" s="6" t="s">
         <v>13</v>
       </c>
     </row>
+    <row r="350" spans="1:23">
+      <c r="R350" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:V340" xr:uid="{CBF823FE-3832-334D-A267-F2D8B0A33CAA}"/>
+  <autoFilter ref="A3:V340"/>
   <mergeCells count="2">
     <mergeCell ref="K2:S2"/>
     <mergeCell ref="U2:V2"/>

</xml_diff>